<commit_message>
feat: add HA, NAT, Objects automation and fix CLI push syntax with IP format
</commit_message>
<xml_diff>
--- a/policies.xlsx
+++ b/policies.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Security_Zones" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="NAT_Policies" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Security_Policies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="HA_Configuration" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,8 +47,20 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -74,8 +87,26 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F9"/>
+        <bgColor rgb="00F2F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -97,11 +128,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D3D3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +162,27 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -533,110 +599,578 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>CORP-LAN</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NET-LAN-Users</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>ip-netmask</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>192.168.10.0/24</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Corporate LAN subnet</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>corp</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>10.10.10.0/24</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Corporate Users &amp; Workstations Subnet</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>DMZ-HOST</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NET-LAN-Servers</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>ip-netmask</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>10.0.0.50/32</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>DMZ web server</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>dmz</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10.10.20.0/24</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Internal Corporate Servers Subnet</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>GUEST-RANGE</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NET-LAN-Mgmt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>10.10.30.0/24</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Network and IT Infrastructure Management Subnet</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NET-VPN-Pool</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>10.10.40.0/24</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Remote Access VPN Client IP Pool</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NET-Mail-Clients</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>10.10.50.0/24</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Internal Mail Clients and SMTP Relays</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NET-DMZ-Servers</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>10.20.20.0/24</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Public-Facing DMZ Server Subnet</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NET-Guest-WiFi</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>10.99.0.0/24</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Isolated Guest Wi-Fi Network</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NET-Database-Farm</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>10.30.30.0/24</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Backend Database Farm Subnet</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HOST-DMZ-Web</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>10.20.20.10/32</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Production DMZ Web Application Server</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HOST-DMZ-Mail</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10.20.20.30/32</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Production DMZ Mail and SMTP Server</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HOST-DB-Server</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10.30.30.20/32</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Production Database Server (MySQL/Oracle)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HOST-Mgmt-Server</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10.10.30.10/32</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Central IT Bastion / Jump Server</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HOST-NMS-Monitoring</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10.10.60.10/32</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Enterprise NMS / Monitoring Host</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PUB-Web-Server-VIP</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>203.0.113.20/32</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>External Public VIP for Inbound Web Traffic</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PUB-Mail-Server-VIP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>203.0.113.25/32</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>External Public VIP for Inbound Mail Traffic</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PUB-PAT-Internet-IP</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ip-netmask</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>203.0.113.10/32</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Public Egress NAT Pool for Corporate Users</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FQDN-PaloAlto-Updates</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>fqdn</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>updates.paloaltonetworks.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Palo Alto Dynamic Content Updates FQDN</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RNG-DHCP-Pool</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>ip-range</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>172.16.0.1-172.16.0.254</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Guest pool</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>guest</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>EXT-API</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>fqdn</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>api.example.com</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>External API endpoint</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>external</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10.10.10.100-10.10.10.200</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Corporate DHCP Client Allocation Pool</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
         </is>
       </c>
     </row>
@@ -651,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -707,118 +1241,322 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TCP-3306</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tcp</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3306</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MySQL / MariaDB Database Service</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>SVC-HTTPS-8443</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>tcp</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>8443</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Custom HTTPS</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>web</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>SVC-DNS-UDP</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Custom Web Administration HTTPS</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SVC-HTTP-8080</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tcp</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8080</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Alternative HTTP Web Proxy / App Server</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SVC-RDP-3389</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tcp</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3389</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Microsoft Remote Desktop Protocol</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SVC-SSH-2222</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tcp</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2222</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Alternate SSH Administration Port</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SVC-MSSQL-1433</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tcp</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1433</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Microsoft SQL Server Database Port</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SVC-SYSLOG-UDP-514</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>udp</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Syslog / SIEM UDP Log Receiver</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SVC-SNMP-UDP-161</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>udp</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SNMP Polling and Monitoring Service</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SVC-NTP-UDP-123</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>udp</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Network Time Protocol Synchronization</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SVC-DNS-UDP-53</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>udp</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>DNS</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>infra</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>SVC-RDP</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>tcp</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>3389</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Remote Desktop</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>mgmt</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>SVC-HTTP-HTTPS</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>tcp-udp</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>80,443</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>1024-65535</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Web combo</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>web</t>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Domain Name System Standard UDP Queries</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
         </is>
       </c>
     </row>
@@ -997,7 +1735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1101,126 +1839,317 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>TRUST-TO-INTERNET-NAT</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>TRUST</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>UNTRUST</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>CORP-LAN</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Inside-Internet-PAT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inside_zone</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10.10.10.0/24, 10.10.20.0/24, 10.10.30.0/24, 10.10.50.0/24</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>any</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>any</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>ipv4</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>dynamic-ip-and-port</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>ethernet1/2</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Outbound NAT for corp</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>nat</t>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>203.0.113.10</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Outbound PAT for internal enterprise subnets to Internet</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>INBOUND-DMZ-DNAT</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>UNTRUST</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>DMZ</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Guest-Internet-PAT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Guest_zone</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10.99.0.0/24</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>any</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>any</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>SVC-HTTPS-8443</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>ipv4</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>dynamic-ip-and-port</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>203.0.113.11</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Outbound PAT for isolated guest Wi-Fi network</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VPN-Outbound-PAT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VPN_zone</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10.10.40.0/24</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ipv4</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>dynamic-ip-and-port</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>203.0.113.12</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Outbound PAT for remote VPN client egress traffic</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DMZ-Web-Server-DNAT</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>203.0.113.20</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>service-https</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ipv4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>10.0.0.50</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>8443</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Port-forward to DMZ server</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>dnat</t>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>10.20.20.10</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>443</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Inbound HTTPS DNAT port forwarding for DMZ web server</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DMZ-Mail-Server-DNAT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Outside_zone</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>203.0.113.25</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ipv4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>10.20.20.30</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Inbound 1-to-1 DNAT forwarding for DMZ mail server</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>FPR2140-MUM-1</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>PUSHED</t>
         </is>
       </c>
     </row>
@@ -1360,12 +2289,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>web-browsing, ssl</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>HTTP,HTTPS</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -1394,11 +2323,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
@@ -1429,12 +2354,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>dns</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1463,11 +2388,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -1498,12 +2419,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>ssl</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1532,11 +2453,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
@@ -1567,12 +2484,12 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>ssh</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>SSH</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -1601,11 +2518,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
@@ -1670,11 +2583,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1739,11 +2648,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1774,12 +2679,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>ntp</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>NTP</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -1808,11 +2713,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1843,12 +2744,12 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>smtp</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>SMTP</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1877,11 +2778,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1946,11 +2843,7 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1981,12 +2874,12 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>any</t>
+          <t>ping</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>ICMP</t>
+          <t>application-default</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -2015,12 +2908,710 @@
           <t>FPR2140-MUM-1</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>DRY-RUN</t>
-        </is>
-      </c>
+      <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="67" customWidth="1" min="6" max="6"/>
+    <col width="95" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Item #</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>HA Component</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Firewall A (Primary / Active)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Firewall B (Secondary / Standby)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Description / Purpose</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>CLI Command (Firewall A)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>CLI Command (Firewall B)</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Deployment Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Global HA</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Enable High Availability state machine on chassis</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability enabled yes</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability enabled yes</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>HA Group</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>group-id</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>HA Cluster Group ID (must match on both peers)</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group group-id 1</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group group-id 1</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>HA Group</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>HA-Pair-Active-Passive</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>HA-Pair-Active-Passive</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Descriptive tag for cluster identifier</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group description HA-Pair-Active-Passive</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group description HA-Pair-Active-Passive</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>HA Group</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>active-passive</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>active-passive</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Operational Mode: Active/Passive failover</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group mode active-passive</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group mode active-passive</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>HA Group</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>peer-ip</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>10.254.1.2</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>10.254.1.1</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>HA1 Peer IPv4 address for control link heartbeats</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group peer-ip 10.254.1.2</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group peer-ip 10.254.1.1</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Election Option</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>device-priority</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>100 (Primary)</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>200 (Secondary)</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Device Priority: lower value indicates preferred active peer</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group election-option device-priority 100</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group election-option device-priority 200</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Election Option</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>preemptive</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Preemption enabled to reclaim Active state upon recovery</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group election-option preemptive yes</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group election-option preemptive yes</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>State Sync</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>state-synchronization</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>enabled yes</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>enabled yes</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Synchronize active sessions, NAT, and IPSec SA states across HA2</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group state-synchronization enabled yes</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability group state-synchronization enabled yes</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>HA1 Interface</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>network interface type</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>ethernet1/3 (ha)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>ethernet1/3 (ha)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Configure ethernet1/3 physical interface for HA link</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>set network interface ethernet ethernet1/3 ha</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>set network interface ethernet ethernet1/3 ha</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>HA1 Interface</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>ha1 port binding</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>ethernet1/3</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>ethernet1/3</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Bind HA1 control link to dedicated ethernet1/3 port</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha1 port ethernet1/3</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha1 port ethernet1/3</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>HA1 Interface</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>ha1 ip-address &amp; netmask</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>10.254.1.1 / 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>10.254.1.2 / 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Point-to-point HA1 Control network /24</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha1 ip-address 10.254.1.1 netmask 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha1 ip-address 10.254.1.2 netmask 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>HA2 Interface</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>network interface type</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>ethernet1/4 (ha)</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>ethernet1/4 (ha)</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Configure ethernet1/4 physical interface for HA link</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>set network interface ethernet ethernet1/4 ha</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>set network interface ethernet ethernet1/4 ha</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>HA2 Interface</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>ha2 port binding</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>ethernet1/4</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>ethernet1/4</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Bind HA2 data/session synchronization link to ethernet1/4 port</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha2 port ethernet1/4</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha2 port ethernet1/4</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>HA2 Interface</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>ha2 ip-address &amp; netmask</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>10.254.2.1 / 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>10.254.2.2 / 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Point-to-point HA2 Data sync network /24</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha2 ip-address 10.254.2.1 netmask 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>set deviceconfig high-availability interface ha2 ip-address 10.254.2.2 netmask 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>COMMITTED</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>